<commit_message>
Add regression analysis: which questionnaire dimensions predict simulation
Multiple OLS regression (N=1223) predicting simulation SRL performance from
6 questionnaire dimensions. R²=0.065. Only מוטיבציה (β=.108*) and
יוזמה ואחריות (β=.106**) are unique significant predictors; others lose
significance due to predictor intercorrelation (r≈.54, VIF 1.6-3.0).

https://claude.ai/code/session_011BCKSU8z4oQR3ER1cBLppb
</commit_message>
<xml_diff>
--- a/ניתוח_מתאם_סימולציה_שאלון.xlsx
+++ b/ניתוח_מתאם_סימולציה_שאלון.xlsx
@@ -11,6 +11,7 @@
     <sheet name="מתאמים לפי ממד" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="מטריצת מתאמים צולבת" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="פרשנות וסיכום" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="רגרסיה - מה מנבא" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -100,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -121,6 +122,15 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1111,9 +1121,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
@@ -1121,9 +1129,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
@@ -1145,9 +1151,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
@@ -1169,9 +1173,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
@@ -1193,9 +1195,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
@@ -1214,6 +1214,283 @@
       <c r="A20" t="inlineStr">
         <is>
           <t xml:space="preserve">   בין מדדי דיווח-עצמי למדדי ביצוע בפועל.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>רגרסיה מרובה: אילו ממדי שאלון מנבאים את הביצוע בסימולציה?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>N = 1223 תלמידים  |  R² = 0.065  (השאלון מנבא 6.5% מהשונות בסימולציה)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>ממד בשאלון</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>β סטנדרטי (תרומה ייחודית)</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>p-value</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>מובהקות</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>r פשוט (קשר ישיר)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>מוטיבציה</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>0.108</v>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>0.0125</v>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>יוזמה ואחריות</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="n">
+        <v>0.106</v>
+      </c>
+      <c r="C6" s="13" t="n">
+        <v>0.0062</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>**</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>0.218</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>תודעת צמיחה</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>0.0988</v>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>0.197</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>מודעות עצמית</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>0.703</v>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>0.168</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>ויסות עצמי</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>0.7994</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>0.199</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>תמיכה רגשית</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>0.8914</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>0.152</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>פרשנות:</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>• β (בטא) = התרומה הייחודית של כל ממד לניבוי, בנטרול שאר הממדים.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>• r פשוט = הקשר הישיר של הממד עם הסימולציה (ללא נטרול).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>ממצא מרכזי: רק שני ממדים מנבאים באופן ייחודי ומובהק את הביצוע בסימולציה:</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   1. מוטיבציה ורלוונטיות (β=0.108, p&lt;.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   2. יוזמה ואחריות (β=0.106, p&lt;.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>שאר הממדים (ויסות, מודעות, תמיכה, צמיחה) מאבדים מובהקות ברגרסיה למרות</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>שיש להם קשר ישיר דומה (r≈0.15-0.20) — כי כוח הניבוי שלהם חופף לזה של</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>מוטיבציה ויוזמה (הממדים בשאלון מתואמים זה לזה ב-r≈0.54).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>מסקנה: 'מוטיבציה' ו'יוזמה ואחריות' הם הליבה המנבאת ביצוע התנהגותי בפועל.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>תלמיד שמדווח על מוטיבציה גבוהה ויוזמה רבה — נוטה להפגין רמות SRL גבוהות בסימולציה.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add AI vs no-AI regression split analysis
Separate OLS regressions by pilot(AI)/comparison(no-AI) group, validated
99.8% against questionnaire group indicator.

Key finding: prediction pattern differs by group.
- No-AI (N=241): R²=0.130, motivation dominant predictor (β=.26**)
- AI (N=979): R²=0.058, initiative dominant (β=.12**), motivation n.s.
AI appears to attenuate the self-report→behavior link.

https://claude.ai/code/session_011BCKSU8z4oQR3ER1cBLppb
</commit_message>
<xml_diff>
--- a/ניתוח_מתאם_סימולציה_שאלון.xlsx
+++ b/ניתוח_מתאם_סימולציה_שאלון.xlsx
@@ -12,6 +12,7 @@
     <sheet name="מטריצת מתאמים צולבת" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="פרשנות וסיכום" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="רגרסיה - מה מנבא" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="פילוח AI מול ללא AI" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,6 +46,11 @@
     <font>
       <i val="1"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="6">
@@ -101,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -130,6 +136,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1121,7 +1130,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
@@ -1129,7 +1137,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
@@ -1151,7 +1158,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
@@ -1173,7 +1179,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
@@ -1195,7 +1200,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
@@ -1405,9 +1409,7 @@
         <v>0.152</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
@@ -1429,9 +1431,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-    </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
@@ -1453,9 +1453,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
@@ -1477,9 +1475,7 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr"/>
-    </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
@@ -1491,6 +1487,333 @@
       <c r="A26" t="inlineStr">
         <is>
           <t>תלמיד שמדווח על מוטיבציה גבוהה ויוזמה רבה — נוטה להפגין רמות SRL גבוהות בסימולציה.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>פילוח רגרסיה: עם AI (פיילוט) מול ללא AI (השוואה)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>🤖 קבוצת AI:  N=979  |  R²=0.058 (5.8% ניבוי)  |  ביצוע ממוצע=2.03</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>📝 קבוצת ללא AI:  N=241  |  R²=0.130 (13.0% ניבוי)  |  ביצוע ממוצע=2.09</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>ממד בשאלון</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>β (AI)</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>מובהקות AI</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>β (ללא AI)</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>מובהקות ללא AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>מוטיבציה</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>0.259</v>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>**</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>תודעת צמיחה</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>0.161</v>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>יוזמה ואחריות</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>**</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>ויסות עצמי</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>-0.148</v>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>מודעות עצמית</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>-0.017</v>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>0.082</v>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>תמיכה רגשית</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>-0.011</v>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>ממצאים מרכזיים:</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>1. כוח הניבוי כפול בקבוצת ללא-AI: R²=13.0% מול 5.8% בלבד בקבוצת ה-AI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   בלי AI — הדיווח העצמי של התלמיד חוזה את ביצועו הרבה יותר טוב.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>2. מנבא שונה בכל קבוצה:</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • ללא AI → מוטיבציה ורלוונטיות הוא המנבא הדומיננטי (β=0.26, p&lt;.01).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • עם AI → יוזמה ואחריות הוא המנבא היחיד המובהק (β=0.12, p&lt;.01);</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     המוטיבציה מאבדת את כוח הניבוי שלה.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>3. פרשנות אפשרית: כלי ה-AI 'מרכך' את הקשר בין מוטיבציה פנימית לביצוע —</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   הוא מספק תמיכה/פיגומים לכל התלמידים ללא קשר למוטיבציה שלהם, ולכן</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   המוטיבציה כבר לא מבדילה בין מצליחים לפחות מצליחים. במקום זה, בולטת</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   היכולת ליזום ולקחת אחריות על השימוש בכלי.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>4. הפרש הביצוע בין הקבוצות זניח מבחינה מעשית (2.03 מול 2.09),</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   אם כי מובהק סטטיסטית (p=.013) בשל המדגם הגדול.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>אזהרה: בקבוצת ללא-AI (N=241) חלק מהמקדמים פחות יציבים בשל מדגם קטן יותר</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>וחפיפה בין המנבאים. הממצא היציב הוא ש-R² גבוה יותר והמוטיבציה דומיננטית.</t>
         </is>
       </c>
     </row>

</xml_diff>